<commit_message>
Uppdaterade figurer för 2026
Behöver se över texten i testet så att det inte finns hänvisningar till data från föregående år.
</commit_message>
<xml_diff>
--- a/data/anställning_sektor.xlsx
+++ b/data/anställning_sektor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://svenskidrott-my.sharepoint.com/personal/william_lind_rfsisu_se/Documents/Dokument/GitHub/svenskstatistik-arbete/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://svenskidrott-my.sharepoint.com/personal/william_lind_rfsisu_se/Documents/Dokument/GitHub/RF-SISU Uppland/sverige-i-siffror/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="11_708ECC4B6DFF70B00DD3870D2033360BC102618E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DEC5F9E-1CF8-4E2E-A1D5-A0CF632699D8}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="11_708ECC4B6DFF70B00DD3870D2033360BC102618E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCEA3E95-8817-46FF-A92D-0D73909F1ADA}"/>
   <bookViews>
-    <workbookView xWindow="31635" yWindow="2415" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0000070M" sheetId="2" r:id="rId1"/>
@@ -426,7 +426,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="2">
-        <v>2839714</v>
+        <v>2774487</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -437,7 +437,7 @@
         <v>9</v>
       </c>
       <c r="C3" s="2">
-        <v>2741253</v>
+        <v>2666351</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -448,7 +448,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="2">
-        <v>5580967</v>
+        <v>5440838</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -459,7 +459,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="2">
-        <v>2258661</v>
+        <v>2195975</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -470,7 +470,7 @@
         <v>9</v>
       </c>
       <c r="C6" s="2">
-        <v>1472435</v>
+        <v>1418736</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -481,7 +481,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="2">
-        <v>3731097</v>
+        <v>3614711</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -492,7 +492,7 @@
         <v>8</v>
       </c>
       <c r="C8" s="2">
-        <v>154057</v>
+        <v>159001</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -503,7 +503,7 @@
         <v>9</v>
       </c>
       <c r="C9" s="2">
-        <v>170363</v>
+        <v>176768</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -514,7 +514,7 @@
         <v>10</v>
       </c>
       <c r="C10" s="2">
-        <v>324421</v>
+        <v>335769</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -525,7 +525,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="2">
-        <v>76691</v>
+        <v>75940</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -536,7 +536,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="2">
-        <v>250477</v>
+        <v>243676</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -547,7 +547,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="2">
-        <v>327169</v>
+        <v>319617</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -558,7 +558,7 @@
         <v>8</v>
       </c>
       <c r="C14" s="2">
-        <v>284026</v>
+        <v>278182</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -569,7 +569,7 @@
         <v>9</v>
       </c>
       <c r="C15" s="2">
-        <v>758069</v>
+        <v>735404</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -580,10 +580,16 @@
         <v>10</v>
       </c>
       <c r="C16" s="2">
-        <v>1042095</v>
+        <v>1013586</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{e782e157-8ece-4105-b8e9-fe1eecbfcd69}" enabled="1" method="Privileged" siteId="{eb5b2d6e-028e-454d-b878-0c055adbeb2a}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>